<commit_message>
docs: 핸드오프 검토 보완 — FLOW-017 + 라우팅 + AI 폴백 단계 + POLICY-VISIBILITY
전체 검토 결과 4가지 보완 포인트 모두 반영. 개발자가 코드 작성 시 결정
못 할 정도로 모호한 항목 0건.

04_유저플로우.md
- FLOW-017 추가: 공유 폴더 가시성 + 공개 할 일 수락 흐름
- Happy Path 2종(작성자/수락자) + 9개 분기 케이스 + 메모 비공개 표시

03_IA.md
- 라우팅 보강: /todos/:id/accept (POST 수락), /acceptances (GET 멤버 목록),
  /occurrences (GET 회차 이력)

05_상세기능명세서.md
- POLICY-AI 단계별 분기: 단건 저장 vs 일괄 import × MVP/v1.x 매트릭스
  명시. 어댑터 인터페이스 추상화 가이드
- POLICY-VISIBILITY 신규: TODO-009/010 공통 정책. 할 일은 visibility
  컬럼, 메모는 항상 private. 작성자가 public→private 전환 시 수락자
  알림 즉시 제거 등 엣지 케이스 풀 명세
- 결정 사항 13~15 추가 (회차별 완료·가시성·수락 모델)
- 변경 이력 v1.1·v1.2 추가

06_API명세서.md
- §10.5 신규: AI 폴백 어댑터 구현 가이드. 시나리오별 우선순위 매트릭스
  + TypeScript 인터페이스 + ai_jobs 테이블 보존 정책

02_PRD.md
- KPI 목표치 보강: 평균 할 일 1.5+, 반복 알림 30%+, 회차별 완료율
  50%+. 공유 폴더 공개 할 일 수락률 신규
- 변경 이력 v1.2 추가

build_qlink_spec.py + xlsx
- POLICY-VISIBILITY 추가 → 목록 52행, 상세 ~224행
- 변경 이력 v1.0 / v1.1 / v1.2 3행
</commit_message>
<xml_diff>
--- a/docs/planning/05_상세기능명세서.xlsx
+++ b/docs/planning/05_상세기능명세서.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2361,7 +2361,7 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>owner/member/viewer + 토큰 7일</t>
+          <t>owner/member/viewer + 토큰 7일 + 멤버 50명</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
@@ -2375,6 +2375,39 @@
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>POLICY-VISIBILITY</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>정책</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>공유 폴더 콘텐츠 가시성</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>할 일 private/public 선택 + 메모 항상 private + 수락 필요 모델</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2390,7 +2423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J222"/>
+  <dimension ref="A1:J226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -7911,6 +7944,121 @@
       <c r="H222" s="3" t="inlineStr"/>
       <c r="I222" s="3" t="inlineStr"/>
       <c r="J222" s="3" t="inlineStr"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="3" t="inlineStr">
+        <is>
+          <t>POLICY-VISIBILITY</t>
+        </is>
+      </c>
+      <c r="B223" s="3" t="inlineStr">
+        <is>
+          <t>정책</t>
+        </is>
+      </c>
+      <c r="C223" s="3" t="inlineStr">
+        <is>
+          <t>공유 폴더 콘텐츠 가시성</t>
+        </is>
+      </c>
+      <c r="D223" s="3" t="inlineStr">
+        <is>
+          <t>설명</t>
+        </is>
+      </c>
+      <c r="E223" s="3" t="inlineStr">
+        <is>
+          <t>공유 폴더 link의 부속 콘텐츠(할 일·메모) 노출 규칙. TODO-009/010 공통 사용</t>
+        </is>
+      </c>
+      <c r="F223" s="3" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G223" s="3" t="inlineStr"/>
+      <c r="H223" s="3" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="I223" s="3" t="inlineStr">
+        <is>
+          <t>기획완료</t>
+        </is>
+      </c>
+      <c r="J223" s="3" t="inlineStr">
+        <is>
+          <t>TODO-009/010 공통 정책. 메모와 할 일의 가시성 규칙이 다름</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="3" t="inlineStr"/>
+      <c r="B224" s="3" t="inlineStr"/>
+      <c r="C224" s="3" t="inlineStr"/>
+      <c r="D224" s="3" t="inlineStr">
+        <is>
+          <t>정책</t>
+        </is>
+      </c>
+      <c r="E224" s="3" t="inlineStr">
+        <is>
+          <t>[할 일] visibility: 'private'(default) | 'public'. 사용자 선택
+[메모] visibility 컬럼 없음. 항상 private. UI에 '🔒 나만 볼 수 있는 내용입니다' 안내
+[작성자 표시] public todo는 멤버에게 '👥 {닉네임}이 공유한 할 일'
+[수락 모델] public todo는 명시적 수락(POST /todos/:id/accept)해야 본인 알림 등록
+[DB 일관성] 메모 public 변경 API 호출은 백엔드 차단(400)</t>
+        </is>
+      </c>
+      <c r="F224" s="3" t="inlineStr"/>
+      <c r="G224" s="3" t="inlineStr"/>
+      <c r="H224" s="3" t="inlineStr"/>
+      <c r="I224" s="3" t="inlineStr"/>
+      <c r="J224" s="3" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="3" t="inlineStr"/>
+      <c r="B225" s="3" t="inlineStr"/>
+      <c r="C225" s="3" t="inlineStr"/>
+      <c r="D225" s="3" t="inlineStr">
+        <is>
+          <t>예외</t>
+        </is>
+      </c>
+      <c r="E225" s="3" t="inlineStr">
+        <is>
+          <t>- 비멤버 조회: 403
+- 자기 todo 수락 시도: UI 비활성, API CONFLICT
+- public→private 전환: 기존 수락자 알림 즉시 제거 + Realtime publish
+- 작성자가 public 삭제: 수락 멤버 알림 일괄 제거 (이중 확인 모달)</t>
+        </is>
+      </c>
+      <c r="F225" s="3" t="inlineStr"/>
+      <c r="G225" s="3" t="inlineStr"/>
+      <c r="H225" s="3" t="inlineStr"/>
+      <c r="I225" s="3" t="inlineStr"/>
+      <c r="J225" s="3" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="3" t="inlineStr"/>
+      <c r="B226" s="3" t="inlineStr"/>
+      <c r="C226" s="3" t="inlineStr"/>
+      <c r="D226" s="3" t="inlineStr">
+        <is>
+          <t>마이그레이션</t>
+        </is>
+      </c>
+      <c r="E226" s="3" t="inlineStr">
+        <is>
+          <t>개인 폴더 → 공유 폴더 전환(SHARE-001) 시 기존 todo 자동 'private'. 사용자가 개별 변경</t>
+        </is>
+      </c>
+      <c r="F226" s="3" t="inlineStr"/>
+      <c r="G226" s="3" t="inlineStr"/>
+      <c r="H226" s="3" t="inlineStr"/>
+      <c r="I226" s="3" t="inlineStr"/>
+      <c r="J226" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -8248,7 +8396,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8314,10 +8462,32 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>결정 12건 반영: 이메일 6자리·게스트 출시 제거(Won't)·AI 폴백(MVP=mock+API키, v1.x=외부세션)·FCM Topic 분배+모바일/PC 채널 분리·비밀번호 변경 시 강제 로그아웃·즉시 hard delete·AWS API Gateway WebSocket·last-write-wins·공유멤버 50명·강조색 3색(핑크/블루/그레이)·단건 외부세션 미사용</t>
+          <t>결정 12건 반영 + 할 일 = 1차 USP 격상: TODO-001~005 Must 추가, 페르소나 시나리오 3개(직장인 PM·취준생·자격증), 다중 할 일·반복 알림(요일+시간) UX, 회차별 완료 + 누적 이력 토글</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>인우</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>v1.0.2</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>공유 폴더 가시성·수락 흐름: TODO-009(할 일 private/public 선택), TODO-010(공개 할 일 수락), POLICY-VISIBILITY 신규, 메모 항상 비공개 + 안내 문구. FLOW-017 추가, 색상 가독성 전면 개선(--qlink-primary 기반)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>인우</t>
         </is>

</xml_diff>